<commit_message>
With period definitions added
</commit_message>
<xml_diff>
--- a/Kate Dale_Honours Dataset_FINAL 29.5.26.xlsx
+++ b/Kate Dale_Honours Dataset_FINAL 29.5.26.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/user/Documents/Honours/Dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{48918BEC-463C-3744-AF03-C56AA706F934}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F459BD61-D799-304D-A2B8-81C5531E9948}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="44800" windowHeight="23000" xr2:uid="{1D74D2EC-D460-0E4F-B015-3F28AF0D107A}"/>
+    <workbookView xWindow="25240" yWindow="520" windowWidth="19560" windowHeight="23000" firstSheet="9" activeTab="12" xr2:uid="{1D74D2EC-D460-0E4F-B015-3F28AF0D107A}"/>
   </bookViews>
   <sheets>
     <sheet name="Dataset Schema" sheetId="2" r:id="rId1"/>
@@ -32,7 +32,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="1" r:id="rId14"/>
+    <pivotCache cacheId="2" r:id="rId14"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6018" uniqueCount="1311">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6040" uniqueCount="1323">
   <si>
     <t>Ceremonial</t>
   </si>
@@ -4215,6 +4215,42 @@
   <si>
     <t xml:space="preserve">Charlie Hippai, Lady Hippai and Peter Hippai
 </t>
+  </si>
+  <si>
+    <t>References  associated with the Dreamtime</t>
+  </si>
+  <si>
+    <t>References associated with an unknown period prior to 1840</t>
+  </si>
+  <si>
+    <t>References associated with the period from 1840-1849</t>
+  </si>
+  <si>
+    <t>References associated with the period from 1850-1859</t>
+  </si>
+  <si>
+    <t>References associated with the period from 1860-1869</t>
+  </si>
+  <si>
+    <t>References associated with the period from 1870-1879</t>
+  </si>
+  <si>
+    <t>References associated with the period from 1880-1889</t>
+  </si>
+  <si>
+    <t>References associated with the period from 1890-1899</t>
+  </si>
+  <si>
+    <t>References associated with the period of 1900</t>
+  </si>
+  <si>
+    <t>References associated with an unknown period between 1840-1900</t>
+  </si>
+  <si>
+    <t>Definitions of periods</t>
+  </si>
+  <si>
+    <t>period Definition</t>
   </si>
 </sst>
 </file>
@@ -4760,7 +4796,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="114">
+  <cellXfs count="117">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -5006,6 +5042,18 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -5024,20 +5072,8 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -5045,6 +5081,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5590,6 +5633,48 @@
           <bgColor theme="0"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -6186,48 +6271,6 @@
           <color indexed="64"/>
         </horizontal>
       </border>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="right"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="right"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -27975,7 +28018,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FF8339C2-F7CA-004E-8E5C-3A7E6B7E2613}" name="PivotTable12" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FF8339C2-F7CA-004E-8E5C-3A7E6B7E2613}" name="PivotTable12" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="B35:X47" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
@@ -28174,7 +28217,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable10.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5D78F90B-4103-B24B-BC63-5828426FA314}" name="PivotTable8" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" grandTotalCaption="Grand Total" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5D78F90B-4103-B24B-BC63-5828426FA314}" name="PivotTable8" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" grandTotalCaption="Grand Total" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="B22:M35" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
@@ -28318,24 +28361,24 @@
     <dataField name="Count of period" fld="11" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="5">
-    <format dxfId="149">
+    <format dxfId="101">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="11" count="0" selected="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="148">
+    <format dxfId="100">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="11" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="147">
+    <format dxfId="99">
       <pivotArea dataOnly="0" grandCol="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="146">
+    <format dxfId="98">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="11" count="1">
@@ -28344,7 +28387,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="145">
+    <format dxfId="97">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="11" count="1">
@@ -28367,8 +28410,8 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable11.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{676D4B45-E5CD-5641-8482-88793E8E33FA}" name="PivotTable6" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="B4:C16" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B437B2B5-1664-2548-85F6-6CECF3005C22}" name="PivotTable7" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
+  <location ref="E4:K17" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
@@ -28387,7 +28430,7 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField axis="axisRow" dataField="1" showAll="0">
+    <pivotField axis="axisRow" showAll="0">
       <items count="12">
         <item x="8"/>
         <item x="5"/>
@@ -28403,7 +28446,18 @@
         <item t="default"/>
       </items>
     </pivotField>
-    <pivotField showAll="0"/>
+    <pivotField axis="axisCol" dataField="1" showAll="0">
+      <items count="8">
+        <item m="1" x="5"/>
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item m="1" x="6"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
@@ -28455,17 +28509,116 @@
       <x/>
     </i>
   </rowItems>
-  <colItems count="1">
-    <i/>
+  <colFields count="1">
+    <field x="18"/>
+  </colFields>
+  <colItems count="6">
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
   </colItems>
   <dataFields count="1">
-    <dataField name="Count of historical_theme" fld="17" subtotal="count" baseField="0" baseItem="0"/>
+    <dataField name="Count of place_category" fld="18" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
-  <formats count="1">
-    <format dxfId="150">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+  <formats count="4">
+    <format dxfId="105">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="18" count="0" selected="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="104">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="18" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="103">
+      <pivotArea grandCol="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="102">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
+  <chartFormats count="5">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="18" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="18" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="18" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="3" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="18" count="1" selected="0">
+            <x v="4"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="4" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="18" count="1" selected="0">
+            <x v="5"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight15" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
@@ -28479,7 +28632,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable12.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3D62713B-9F8A-E840-BABA-5B517B1740F0}" name="PivotTable2" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="18">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3D62713B-9F8A-E840-BABA-5B517B1740F0}" name="PivotTable2" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="18">
   <location ref="A4:C10" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -28639,7 +28792,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable13.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{EB548357-F74C-8444-A768-CDAE66F1A87F}" name="PivotTable1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="5">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{EB548357-F74C-8444-A768-CDAE66F1A87F}" name="PivotTable1" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="5">
   <location ref="A15:C21" firstHeaderRow="1" firstDataRow="1" firstDataCol="2"/>
   <pivotFields count="28">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -29357,7 +29510,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable14.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{431073AF-99BD-6544-A074-24A523B00CC8}" name="PivotTable4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" grandTotalCaption="Total" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="place_type">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{431073AF-99BD-6544-A074-24A523B00CC8}" name="PivotTable4" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" grandTotalCaption="Total" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="place_type">
   <location ref="B41:C45" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
@@ -29433,7 +29586,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable15.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E5D8018C-5317-064F-9916-EA9F94B674AB}" name="PivotTable3" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" grandTotalCaption="Total" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="place_type">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E5D8018C-5317-064F-9916-EA9F94B674AB}" name="PivotTable3" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" grandTotalCaption="Total" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="place_type">
   <location ref="B30:C37" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
@@ -29522,7 +29675,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable16.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00DFF08D-0B6E-6448-93FD-25831A6C2E07}" name="PivotTable2" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" grandTotalCaption="Total" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="place_type">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00DFF08D-0B6E-6448-93FD-25831A6C2E07}" name="PivotTable2" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" grandTotalCaption="Total" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="place_type">
   <location ref="B4:C26" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
@@ -29677,7 +29830,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable17.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A028AB9E-24FA-BC4C-9317-2B89AD171D85}" name="PivotTable17" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A028AB9E-24FA-BC4C-9317-2B89AD171D85}" name="PivotTable17" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A43:E48" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
@@ -29802,7 +29955,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable18.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{57812AA5-A583-8741-B532-B773D261C6C4}" name="PivotTable16" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{57812AA5-A583-8741-B532-B773D261C6C4}" name="PivotTable16" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A31:E39" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
@@ -29940,7 +30093,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable19.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3A250399-2A38-E74C-867B-89C57BE24D3D}" name="PivotTable5" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="4">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3A250399-2A38-E74C-867B-89C57BE24D3D}" name="PivotTable5" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="4">
   <location ref="A4:G27" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -30150,7 +30303,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D34AB9AC-D393-AD42-B429-1C5FBD2BDAA6}" name="PivotTable11" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="25">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D34AB9AC-D393-AD42-B429-1C5FBD2BDAA6}" name="PivotTable11" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="25">
   <location ref="B20:H32" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
@@ -30272,14 +30425,14 @@
     <dataField name="Count of place_category" fld="18" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="101">
+    <format dxfId="115">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="18" count="0" selected="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="100">
+    <format dxfId="114">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="18" count="0"/>
@@ -30482,7 +30635,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable20.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3FAC62E4-CE0E-B448-B0AD-E9DAFC687FCC}" name="PivotTable1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3FAC62E4-CE0E-B448-B0AD-E9DAFC687FCC}" name="PivotTable1" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A4:B88" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -31051,7 +31204,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable21.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{DC2A81C9-2295-5D4A-9D9E-67042CBE96DD}" name="PivotTable5" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{DC2A81C9-2295-5D4A-9D9E-67042CBE96DD}" name="PivotTable5" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="G4:H93" firstHeaderRow="1" firstDataRow="1" firstDataCol="2"/>
   <pivotFields count="28">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -31712,7 +31865,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable22.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{398DAB95-6B62-7542-991E-CC0B1911D56D}" name="PivotTable23" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="8" rowHeaderCaption="Ranking of coordinates precision">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{398DAB95-6B62-7542-991E-CC0B1911D56D}" name="PivotTable23" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="8" rowHeaderCaption="Ranking of coordinates precision">
   <location ref="B4:C9" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
@@ -31926,7 +32079,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable23.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{AF72CEC9-EB7F-CB4B-8771-70A8FC1B66DB}" name="PivotTable21" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{AF72CEC9-EB7F-CB4B-8771-70A8FC1B66DB}" name="PivotTable21" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
   <location ref="J4:O10" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
@@ -32291,7 +32444,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable24.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E7EF111F-433C-0D40-9BBB-6138C0E23072}" name="PivotTable2" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" grandTotalCaption="Total" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1" rowHeaderCaption="(filter on place_name)" colHeaderCaption="">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E7EF111F-433C-0D40-9BBB-6138C0E23072}" name="PivotTable2" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" grandTotalCaption="Total" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1" rowHeaderCaption="(filter on place_name)" colHeaderCaption="">
   <location ref="A3:G88" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
@@ -32778,7 +32931,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable25.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{755CB6A8-F227-BD4A-8C6B-B14AD47B09EF}" name="PivotTable1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{755CB6A8-F227-BD4A-8C6B-B14AD47B09EF}" name="PivotTable1" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A2:M87" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
@@ -33269,7 +33422,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5B06BAFF-02CC-6045-8A5D-C7221D3A1BEA}" name="PivotTable10" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5B06BAFF-02CC-6045-8A5D-C7221D3A1BEA}" name="PivotTable10" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="B80:N92" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
@@ -33413,7 +33566,7 @@
     <dataField name="Count of place_category" fld="18" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="102">
+    <format dxfId="116">
       <pivotArea dataOnly="0" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="17" count="0"/>
@@ -33434,7 +33587,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{866A254B-AD3F-2D41-9122-CB764CF3D95B}" name="PivotTable2" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="14">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{866A254B-AD3F-2D41-9122-CB764CF3D95B}" name="PivotTable2" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="14">
   <location ref="B4:C15" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
@@ -33566,229 +33719,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B437B2B5-1664-2548-85F6-6CECF3005C22}" name="PivotTable7" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
-  <location ref="E4:K17" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="28">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="12">
-        <item x="8"/>
-        <item x="5"/>
-        <item x="0"/>
-        <item x="6"/>
-        <item x="1"/>
-        <item x="10"/>
-        <item x="9"/>
-        <item x="2"/>
-        <item x="7"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisCol" dataField="1" showAll="0">
-      <items count="8">
-        <item m="1" x="5"/>
-        <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="4"/>
-        <item x="3"/>
-        <item m="1" x="6"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="17"/>
-  </rowFields>
-  <rowItems count="12">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i>
-      <x v="10"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="18"/>
-  </colFields>
-  <colItems count="6">
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Count of place_category" fld="18" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <formats count="4">
-    <format dxfId="140">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
-        <references count="1">
-          <reference field="18" count="0" selected="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="139">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="18" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="138">
-      <pivotArea grandCol="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="137">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="5">
-    <chartFormat chart="0" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="18" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="1" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="18" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="18" count="1" selected="0">
-            <x v="3"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="3" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="18" count="1" selected="0">
-            <x v="4"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="4" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="18" count="1" selected="0">
-            <x v="5"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight15" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{40E5F6EB-967C-394A-BAD8-4CA202DEDFD9}" name="PivotTable14" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{40E5F6EB-967C-394A-BAD8-4CA202DEDFD9}" name="PivotTable14" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="B74:N97" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
@@ -33979,14 +33910,14 @@
     <dataField name="Count of place_type_1" fld="19" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="142">
+    <format dxfId="93">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="17" count="0" selected="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="141">
+    <format dxfId="92">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="17" count="0"/>
@@ -34006,8 +33937,120 @@
 </pivotTableDefinition>
 </file>
 
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{676D4B45-E5CD-5641-8482-88793E8E33FA}" name="PivotTable6" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="B4:C16" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="28">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" dataField="1" showAll="0">
+      <items count="12">
+        <item x="8"/>
+        <item x="5"/>
+        <item x="0"/>
+        <item x="6"/>
+        <item x="1"/>
+        <item x="10"/>
+        <item x="9"/>
+        <item x="2"/>
+        <item x="7"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="17"/>
+  </rowFields>
+  <rowItems count="12">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of historical_theme" fld="17" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="1">
+    <format dxfId="94">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight15" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
 <file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{7F76D8A8-3873-CE44-9B15-DC7D401C95D2}" name="PivotTable1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="24">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{7F76D8A8-3873-CE44-9B15-DC7D401C95D2}" name="PivotTable1" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="24">
   <location ref="O4:P16" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
@@ -34102,10 +34145,10 @@
     <dataField name="% of historical_theme" fld="17" subtotal="count" showDataAs="percentOfTotal" baseField="0" baseItem="0" numFmtId="10"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="144">
+    <format dxfId="96">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="143">
+    <format dxfId="95">
       <pivotArea outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -34412,7 +34455,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A35914F5-E8F2-9942-90D9-D73227088057}" name="PivotTable5" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A35914F5-E8F2-9942-90D9-D73227088057}" name="PivotTable5" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="B38:M45" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
@@ -34546,7 +34589,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable9.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{83629486-73F7-2B4A-B03B-54E32B8FB999}" name="PivotTable9" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{83629486-73F7-2B4A-B03B-54E32B8FB999}" name="PivotTable9" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="B48:M71" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
@@ -34745,19 +34788,19 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{181B682D-CF76-8540-A5A1-021E46289E18}" name="Table2" displayName="Table2" ref="A3:C25" totalsRowShown="0" headerRowDxfId="136" headerRowBorderDxfId="135" tableBorderDxfId="134" totalsRowBorderDxfId="133">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{181B682D-CF76-8540-A5A1-021E46289E18}" name="Table2" displayName="Table2" ref="A3:C25" totalsRowShown="0" headerRowDxfId="150" headerRowBorderDxfId="149" tableBorderDxfId="148" totalsRowBorderDxfId="147">
   <autoFilter ref="A3:C25" xr:uid="{181B682D-CF76-8540-A5A1-021E46289E18}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{DFD894FC-56B0-4A41-9D48-D4981FCD8BFD}" name="Field Name" dataDxfId="132"/>
-    <tableColumn id="2" xr3:uid="{E4BF2319-5F64-9F46-B6F6-09580A258867}" name="Definition" dataDxfId="131"/>
-    <tableColumn id="3" xr3:uid="{F8C966A3-DB06-1A4D-B52D-24ACF64A9E29}" name="Type" dataDxfId="130"/>
+    <tableColumn id="1" xr3:uid="{DFD894FC-56B0-4A41-9D48-D4981FCD8BFD}" name="Field Name" dataDxfId="146"/>
+    <tableColumn id="2" xr3:uid="{E4BF2319-5F64-9F46-B6F6-09580A258867}" name="Definition" dataDxfId="145"/>
+    <tableColumn id="3" xr3:uid="{F8C966A3-DB06-1A4D-B52D-24ACF64A9E29}" name="Type" dataDxfId="144"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{05CF9090-EB81-2348-AD89-CC2DE4FD2B53}" name="Table311" displayName="Table311" ref="F2:I25" totalsRowShown="0" headerRowDxfId="129" tableBorderDxfId="128">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{05CF9090-EB81-2348-AD89-CC2DE4FD2B53}" name="Table311" displayName="Table311" ref="F2:I25" totalsRowShown="0" headerRowDxfId="143" tableBorderDxfId="142">
   <autoFilter ref="F2:I25" xr:uid="{05CF9090-EB81-2348-AD89-CC2DE4FD2B53}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{90E32909-E66B-1A47-AD82-B87964E5B4ED}" name="place_category"/>
@@ -34770,7 +34813,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{D5A3D5A5-93BC-514D-A8DF-12F661E1371A}" name="Table412" displayName="Table412" ref="K2:L5" totalsRowShown="0" headerRowDxfId="127" tableBorderDxfId="126">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{D5A3D5A5-93BC-514D-A8DF-12F661E1371A}" name="Table412" displayName="Table412" ref="K2:L5" totalsRowShown="0" headerRowDxfId="141" tableBorderDxfId="140">
   <autoFilter ref="K2:L5" xr:uid="{D5A3D5A5-93BC-514D-A8DF-12F661E1371A}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{910E38D8-0285-1E43-8E9D-9CF331E9099C}" name="Ranking"/>
@@ -34781,45 +34824,45 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{F51A2335-0CA1-4340-95B4-7385526C39A3}" name="Table7" displayName="Table7" ref="A1:V307" totalsRowShown="0" headerRowDxfId="125" dataDxfId="124">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{F51A2335-0CA1-4340-95B4-7385526C39A3}" name="Table7" displayName="Table7" ref="A1:V307" totalsRowShown="0" headerRowDxfId="139" dataDxfId="138">
   <autoFilter ref="A1:V307" xr:uid="{F51A2335-0CA1-4340-95B4-7385526C39A3}"/>
   <tableColumns count="22">
-    <tableColumn id="1" xr3:uid="{01F773ED-3365-BB46-8EAB-416A4527DCA9}" name="identifier" dataDxfId="123"/>
+    <tableColumn id="1" xr3:uid="{01F773ED-3365-BB46-8EAB-416A4527DCA9}" name="identifier" dataDxfId="137"/>
     <tableColumn id="2" xr3:uid="{8ED5562E-77DA-D941-BF5B-CFFA5A7496A0}" name="source_document"/>
-    <tableColumn id="3" xr3:uid="{65F00CBD-CCF2-7348-A20F-9258E59D7E6A}" name="author_surname" dataDxfId="122"/>
-    <tableColumn id="4" xr3:uid="{6EA2009D-E350-C24E-A496-0033744B0F86}" name="author_firstname" dataDxfId="121"/>
-    <tableColumn id="20" xr3:uid="{17E5F703-1BAF-AA4D-BD2B-D8BDDE0E4E26}" name="published_in" dataDxfId="120"/>
-    <tableColumn id="5" xr3:uid="{66FB13E5-DFF7-B446-9A55-A3948A5E3614}" name="year_published" dataDxfId="119"/>
-    <tableColumn id="6" xr3:uid="{49E0CD3E-875A-D54E-B2CF-05639918FC82}" name="page_number" dataDxfId="118"/>
-    <tableColumn id="7" xr3:uid="{CD1C35DD-56E0-0A4A-A95E-A31339256CDD}" name="file_location" dataDxfId="117"/>
-    <tableColumn id="8" xr3:uid="{E49CB8CE-F920-4248-82E0-E7EC616AEBDE}" name="source_document_quote" dataDxfId="116"/>
-    <tableColumn id="9" xr3:uid="{83FB5FAC-00B2-ED44-92C8-1F0A633DA91C}" name="notes" dataDxfId="115"/>
-    <tableColumn id="10" xr3:uid="{C441D23C-1CE6-CB41-9581-4FD3E271A37D}" name="year" dataDxfId="114"/>
-    <tableColumn id="22" xr3:uid="{66F1D9A7-7223-1445-BE42-8F1DD8DCC1FF}" name="period" dataDxfId="113"/>
-    <tableColumn id="11" xr3:uid="{3E22677D-5C88-ED40-944F-C5285234D929}" name="place_name" dataDxfId="112"/>
-    <tableColumn id="12" xr3:uid="{A106FD38-1971-9248-9E0D-F06977FCFC2D}" name="latitude" dataDxfId="111"/>
-    <tableColumn id="13" xr3:uid="{EBD0B98D-A47E-8A40-92AA-442B208BA992}" name="longitude" dataDxfId="110"/>
-    <tableColumn id="14" xr3:uid="{EFF0409A-1228-9C4A-B03A-163C14FDDCFA}" name="coordinates_from" dataDxfId="109"/>
-    <tableColumn id="15" xr3:uid="{FF339948-0558-3D4D-A7EA-60271A9DDDC9}" name="coordinates_precision" dataDxfId="108"/>
-    <tableColumn id="21" xr3:uid="{2975E994-C26C-224A-9BC7-04134A1D44E0}" name="historical_theme" dataDxfId="107"/>
-    <tableColumn id="16" xr3:uid="{299EB9CA-CEA4-284F-B748-C29E05B65B20}" name="place_category" dataDxfId="106"/>
-    <tableColumn id="17" xr3:uid="{5BE448CF-E57A-B247-A30F-3ACC39775DBD}" name="place_type_1" dataDxfId="105"/>
-    <tableColumn id="18" xr3:uid="{158002BC-0F4F-184C-8EFA-6B20890AF4FD}" name="place_type_2" dataDxfId="104"/>
-    <tableColumn id="19" xr3:uid="{C3A6E86A-D72C-5147-819E-BBD50A85BE87}" name="place_type_3" dataDxfId="103"/>
+    <tableColumn id="3" xr3:uid="{65F00CBD-CCF2-7348-A20F-9258E59D7E6A}" name="author_surname" dataDxfId="136"/>
+    <tableColumn id="4" xr3:uid="{6EA2009D-E350-C24E-A496-0033744B0F86}" name="author_firstname" dataDxfId="135"/>
+    <tableColumn id="20" xr3:uid="{17E5F703-1BAF-AA4D-BD2B-D8BDDE0E4E26}" name="published_in" dataDxfId="134"/>
+    <tableColumn id="5" xr3:uid="{66FB13E5-DFF7-B446-9A55-A3948A5E3614}" name="year_published" dataDxfId="133"/>
+    <tableColumn id="6" xr3:uid="{49E0CD3E-875A-D54E-B2CF-05639918FC82}" name="page_number" dataDxfId="132"/>
+    <tableColumn id="7" xr3:uid="{CD1C35DD-56E0-0A4A-A95E-A31339256CDD}" name="file_location" dataDxfId="131"/>
+    <tableColumn id="8" xr3:uid="{E49CB8CE-F920-4248-82E0-E7EC616AEBDE}" name="source_document_quote" dataDxfId="130"/>
+    <tableColumn id="9" xr3:uid="{83FB5FAC-00B2-ED44-92C8-1F0A633DA91C}" name="notes" dataDxfId="129"/>
+    <tableColumn id="10" xr3:uid="{C441D23C-1CE6-CB41-9581-4FD3E271A37D}" name="year" dataDxfId="128"/>
+    <tableColumn id="22" xr3:uid="{66F1D9A7-7223-1445-BE42-8F1DD8DCC1FF}" name="period" dataDxfId="127"/>
+    <tableColumn id="11" xr3:uid="{3E22677D-5C88-ED40-944F-C5285234D929}" name="place_name" dataDxfId="126"/>
+    <tableColumn id="12" xr3:uid="{A106FD38-1971-9248-9E0D-F06977FCFC2D}" name="latitude" dataDxfId="125"/>
+    <tableColumn id="13" xr3:uid="{EBD0B98D-A47E-8A40-92AA-442B208BA992}" name="longitude" dataDxfId="124"/>
+    <tableColumn id="14" xr3:uid="{EFF0409A-1228-9C4A-B03A-163C14FDDCFA}" name="coordinates_from" dataDxfId="123"/>
+    <tableColumn id="15" xr3:uid="{FF339948-0558-3D4D-A7EA-60271A9DDDC9}" name="coordinates_precision" dataDxfId="122"/>
+    <tableColumn id="21" xr3:uid="{2975E994-C26C-224A-9BC7-04134A1D44E0}" name="historical_theme" dataDxfId="121"/>
+    <tableColumn id="16" xr3:uid="{299EB9CA-CEA4-284F-B748-C29E05B65B20}" name="place_category" dataDxfId="120"/>
+    <tableColumn id="17" xr3:uid="{5BE448CF-E57A-B247-A30F-3ACC39775DBD}" name="place_type_1" dataDxfId="119"/>
+    <tableColumn id="18" xr3:uid="{158002BC-0F4F-184C-8EFA-6B20890AF4FD}" name="place_type_2" dataDxfId="118"/>
+    <tableColumn id="19" xr3:uid="{C3A6E86A-D72C-5147-819E-BBD50A85BE87}" name="place_type_3" dataDxfId="117"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8E72A31C-FD9A-CE48-84FE-30CC298C79AD}" name="Table1" displayName="Table1" ref="B50:G61" totalsRowShown="0" headerRowDxfId="99" dataDxfId="98">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8E72A31C-FD9A-CE48-84FE-30CC298C79AD}" name="Table1" displayName="Table1" ref="B50:G61" totalsRowShown="0" headerRowDxfId="113" dataDxfId="112">
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{69D18637-0091-D24F-99F7-A0C712677294}" name="Time Period" dataDxfId="97"/>
-    <tableColumn id="2" xr3:uid="{6707FC34-B078-5749-95E9-2F6C2A820652}" name="Aboriginal Community" dataDxfId="96"/>
-    <tableColumn id="3" xr3:uid="{24A63887-816F-9A47-9E9E-99E4950724D2}" name="Autonomous" dataDxfId="95"/>
-    <tableColumn id="4" xr3:uid="{D81FAB96-C771-7A48-9686-CDEC6F866333}" name="Mission/Reserve" dataDxfId="94"/>
-    <tableColumn id="5" xr3:uid="{5CBF68EF-FD2B-1448-B169-66C604736EBC}" name="Pastoral" dataDxfId="93"/>
-    <tableColumn id="6" xr3:uid="{8DFC3C6E-6FBA-F446-B5D8-EA135D6F325C}" name="Total" dataDxfId="92">
+    <tableColumn id="1" xr3:uid="{69D18637-0091-D24F-99F7-A0C712677294}" name="Time Period" dataDxfId="111"/>
+    <tableColumn id="2" xr3:uid="{6707FC34-B078-5749-95E9-2F6C2A820652}" name="Aboriginal Community" dataDxfId="110"/>
+    <tableColumn id="3" xr3:uid="{24A63887-816F-9A47-9E9E-99E4950724D2}" name="Autonomous" dataDxfId="109"/>
+    <tableColumn id="4" xr3:uid="{D81FAB96-C771-7A48-9686-CDEC6F866333}" name="Mission/Reserve" dataDxfId="108"/>
+    <tableColumn id="5" xr3:uid="{5CBF68EF-FD2B-1448-B169-66C604736EBC}" name="Pastoral" dataDxfId="107"/>
+    <tableColumn id="6" xr3:uid="{8DFC3C6E-6FBA-F446-B5D8-EA135D6F325C}" name="Total" dataDxfId="106">
       <calculatedColumnFormula>SUM(Table1[[#This Row],[Aboriginal Community]:[Pastoral]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -41255,12 +41298,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{042137F7-B753-BB41-96E3-3E4F9847B7AE}">
-  <dimension ref="B1:L25"/>
+  <dimension ref="B1:L31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.33203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="50" customWidth="1"/>
+    <col min="2" max="2" width="17.1640625" customWidth="1"/>
+    <col min="3" max="3" width="57.1640625" customWidth="1"/>
     <col min="4" max="4" width="61.33203125" customWidth="1"/>
     <col min="5" max="5" width="3.6640625" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
@@ -41273,21 +41316,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:12" ht="20" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="104" t="s">
+      <c r="B1" s="108" t="s">
         <v>1095</v>
       </c>
-      <c r="C1" s="105"/>
-      <c r="D1" s="106"/>
-      <c r="F1" s="101" t="s">
+      <c r="C1" s="109"/>
+      <c r="D1" s="110"/>
+      <c r="F1" s="105" t="s">
         <v>236</v>
       </c>
-      <c r="G1" s="102"/>
-      <c r="H1" s="102"/>
-      <c r="I1" s="102"/>
-      <c r="K1" s="101" t="s">
+      <c r="G1" s="106"/>
+      <c r="H1" s="106"/>
+      <c r="I1" s="106"/>
+      <c r="K1" s="105" t="s">
         <v>578</v>
       </c>
-      <c r="L1" s="103"/>
+      <c r="L1" s="107"/>
     </row>
     <row r="2" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B2" s="70" t="s">
@@ -41348,13 +41391,13 @@
       </c>
     </row>
     <row r="4" spans="2:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="109" t="s">
+      <c r="B4" s="101" t="s">
         <v>1138</v>
       </c>
-      <c r="C4" s="108" t="s">
+      <c r="C4" s="111" t="s">
         <v>1277</v>
       </c>
-      <c r="D4" s="107" t="s">
+      <c r="D4" s="103" t="s">
         <v>1185</v>
       </c>
       <c r="F4" s="31"/>
@@ -41373,9 +41416,9 @@
       </c>
     </row>
     <row r="5" spans="2:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="109"/>
-      <c r="C5" s="108"/>
-      <c r="D5" s="107"/>
+      <c r="B5" s="101"/>
+      <c r="C5" s="111"/>
+      <c r="D5" s="103"/>
       <c r="F5" s="31"/>
       <c r="G5" s="31"/>
       <c r="H5" s="31" t="s">
@@ -41392,9 +41435,9 @@
       </c>
     </row>
     <row r="6" spans="2:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="109"/>
-      <c r="C6" s="108"/>
-      <c r="D6" s="107"/>
+      <c r="B6" s="101"/>
+      <c r="C6" s="111"/>
+      <c r="D6" s="103"/>
       <c r="F6" s="31"/>
       <c r="G6" s="31"/>
       <c r="H6" s="31" t="s">
@@ -41508,13 +41551,13 @@
       </c>
     </row>
     <row r="12" spans="2:12" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="109" t="s">
+      <c r="B12" s="101" t="s">
         <v>1151</v>
       </c>
-      <c r="C12" s="110" t="s">
+      <c r="C12" s="102" t="s">
         <v>1283</v>
       </c>
-      <c r="D12" s="107" t="s">
+      <c r="D12" s="103" t="s">
         <v>1244</v>
       </c>
       <c r="F12" s="34" t="s">
@@ -41531,9 +41574,9 @@
       </c>
     </row>
     <row r="13" spans="2:12" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="109"/>
-      <c r="C13" s="110"/>
-      <c r="D13" s="107"/>
+      <c r="B13" s="101"/>
+      <c r="C13" s="102"/>
+      <c r="D13" s="103"/>
       <c r="F13" s="50" t="s">
         <v>3</v>
       </c>
@@ -41548,13 +41591,13 @@
       </c>
     </row>
     <row r="14" spans="2:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="111" t="s">
+      <c r="B14" s="104" t="s">
         <v>1139</v>
       </c>
-      <c r="C14" s="110" t="s">
+      <c r="C14" s="102" t="s">
         <v>1284</v>
       </c>
-      <c r="D14" s="107" t="s">
+      <c r="D14" s="103" t="s">
         <v>1241</v>
       </c>
       <c r="F14" s="28" t="s">
@@ -41571,9 +41614,9 @@
       </c>
     </row>
     <row r="15" spans="2:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="111"/>
-      <c r="C15" s="110"/>
-      <c r="D15" s="107"/>
+      <c r="B15" s="104"/>
+      <c r="C15" s="102"/>
+      <c r="D15" s="103"/>
       <c r="F15" s="28"/>
       <c r="G15" s="28"/>
       <c r="H15" s="28" t="s">
@@ -41641,7 +41684,11 @@
         <v>614</v>
       </c>
     </row>
-    <row r="20" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="114" t="s">
+        <v>1321</v>
+      </c>
+      <c r="C20" s="114"/>
       <c r="F20" s="28"/>
       <c r="G20" s="28"/>
       <c r="H20" s="28" t="s">
@@ -41652,6 +41699,12 @@
       </c>
     </row>
     <row r="21" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B21" s="116" t="s">
+        <v>261</v>
+      </c>
+      <c r="C21" s="116" t="s">
+        <v>1322</v>
+      </c>
       <c r="F21" s="28"/>
       <c r="G21" s="28"/>
       <c r="H21" s="28" t="s">
@@ -41662,6 +41715,12 @@
       </c>
     </row>
     <row r="22" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B22" s="115" t="s">
+        <v>262</v>
+      </c>
+      <c r="C22" s="25" t="s">
+        <v>1311</v>
+      </c>
       <c r="F22" s="28"/>
       <c r="G22" s="28"/>
       <c r="H22" s="28" t="s">
@@ -41672,6 +41731,12 @@
       </c>
     </row>
     <row r="23" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B23" s="115" t="s">
+        <v>1256</v>
+      </c>
+      <c r="C23" s="25" t="s">
+        <v>1312</v>
+      </c>
       <c r="F23" s="28"/>
       <c r="G23" s="28"/>
       <c r="H23" s="28" t="s">
@@ -41682,6 +41747,12 @@
       </c>
     </row>
     <row r="24" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B24" s="115" t="s">
+        <v>1194</v>
+      </c>
+      <c r="C24" s="25" t="s">
+        <v>1313</v>
+      </c>
       <c r="F24" s="28"/>
       <c r="G24" s="28"/>
       <c r="H24" s="28" t="s">
@@ -41692,6 +41763,12 @@
       </c>
     </row>
     <row r="25" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B25" s="115" t="s">
+        <v>1189</v>
+      </c>
+      <c r="C25" s="25" t="s">
+        <v>1314</v>
+      </c>
       <c r="F25" s="28"/>
       <c r="G25" s="28"/>
       <c r="H25" s="28" t="s">
@@ -41701,17 +41778,60 @@
         <v>621</v>
       </c>
     </row>
+    <row r="26" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B26" s="115" t="s">
+        <v>1190</v>
+      </c>
+      <c r="C26" s="25" t="s">
+        <v>1315</v>
+      </c>
+    </row>
+    <row r="27" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B27" s="115" t="s">
+        <v>1192</v>
+      </c>
+      <c r="C27" s="25" t="s">
+        <v>1316</v>
+      </c>
+    </row>
+    <row r="28" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B28" s="115" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C28" s="25" t="s">
+        <v>1317</v>
+      </c>
+    </row>
+    <row r="29" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B29" s="115" t="s">
+        <v>1191</v>
+      </c>
+      <c r="C29" s="25" t="s">
+        <v>1318</v>
+      </c>
+    </row>
+    <row r="30" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B30" s="115">
+        <v>1900</v>
+      </c>
+      <c r="C30" s="25" t="s">
+        <v>1319</v>
+      </c>
+    </row>
+    <row r="31" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B31" s="115" t="s">
+        <v>1197</v>
+      </c>
+      <c r="C31" s="25" t="s">
+        <v>1320</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:D15">
     <sortCondition ref="B3:B15"/>
   </sortState>
-  <mergeCells count="13">
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="D12:D13"/>
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="B14:B15"/>
+  <mergeCells count="14">
+    <mergeCell ref="B20:C20"/>
     <mergeCell ref="F1:I1"/>
     <mergeCell ref="K1:L1"/>
     <mergeCell ref="K7:L7"/>
@@ -41719,6 +41839,12 @@
     <mergeCell ref="D4:D6"/>
     <mergeCell ref="C4:C6"/>
     <mergeCell ref="B4:B6"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="B14:B15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
Updated time period data
</commit_message>
<xml_diff>
--- a/Kate Dale_Honours Dataset_FINAL 29.5.26.xlsx
+++ b/Kate Dale_Honours Dataset_FINAL 29.5.26.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F459BD61-D799-304D-A2B8-81C5531E9948}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25240" yWindow="520" windowWidth="19560" windowHeight="23000" firstSheet="9" activeTab="12" xr2:uid="{1D74D2EC-D460-0E4F-B015-3F28AF0D107A}"/>
+    <workbookView xWindow="25240" yWindow="500" windowWidth="19560" windowHeight="23000" activeTab="1" xr2:uid="{1D74D2EC-D460-0E4F-B015-3F28AF0D107A}"/>
   </bookViews>
   <sheets>
     <sheet name="Dataset Schema" sheetId="2" r:id="rId1"/>
@@ -32,7 +32,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="2" r:id="rId14"/>
+    <pivotCache cacheId="4" r:id="rId14"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -5030,6 +5030,13 @@
     <xf numFmtId="0" fontId="6" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -5042,17 +5049,8 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -5072,22 +5070,24 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5527,29 +5527,6 @@
       <alignment horizontal="right"/>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <alignment horizontal="right"/>
-    </dxf>
-    <dxf>
       <border>
         <bottom/>
       </border>
@@ -5635,13 +5612,39 @@
       </fill>
     </dxf>
     <dxf>
-      <alignment horizontal="center"/>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
     </dxf>
     <dxf>
       <alignment horizontal="center"/>
     </dxf>
     <dxf>
-      <alignment wrapText="1"/>
+      <alignment horizontal="center"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="14" formatCode="0.00%"/>
@@ -5665,16 +5668,13 @@
       <alignment horizontal="center"/>
     </dxf>
     <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="right"/>
+      <alignment horizontal="center"/>
     </dxf>
     <dxf>
       <alignment horizontal="center"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center"/>
+      <alignment wrapText="1"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -28018,7 +28018,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FF8339C2-F7CA-004E-8E5C-3A7E6B7E2613}" name="PivotTable12" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FF8339C2-F7CA-004E-8E5C-3A7E6B7E2613}" name="PivotTable12" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="B35:X47" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
@@ -28217,8 +28217,8 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable10.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5D78F90B-4103-B24B-BC63-5828426FA314}" name="PivotTable8" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" grandTotalCaption="Grand Total" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
-  <location ref="B22:M35" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{40E5F6EB-967C-394A-BAD8-4CA202DEDFD9}" name="PivotTable14" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="B74:N97" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
@@ -28231,27 +28231,232 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField axis="axisCol" dataField="1" showAll="0">
-      <items count="11">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="12">
+        <item x="8"/>
         <item x="5"/>
+        <item x="0"/>
         <item x="6"/>
+        <item x="1"/>
+        <item x="10"/>
+        <item x="9"/>
+        <item x="2"/>
+        <item x="7"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" dataField="1" showAll="0">
+      <items count="25">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="4"/>
+        <item x="6"/>
+        <item m="1" x="21"/>
+        <item x="18"/>
+        <item x="13"/>
         <item x="7"/>
         <item x="8"/>
+        <item x="17"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="16"/>
         <item x="9"/>
-        <item x="4"/>
+        <item x="3"/>
+        <item x="14"/>
+        <item x="5"/>
         <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item n="Unknown _x000a_1840-1900_x000a_" x="3"/>
+        <item x="10"/>
+        <item x="19"/>
+        <item m="1" x="22"/>
+        <item x="15"/>
+        <item x="20"/>
+        <item m="1" x="23"/>
         <item t="default"/>
       </items>
     </pivotField>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
+    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="19"/>
+  </rowFields>
+  <rowItems count="22">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i>
+      <x v="14"/>
+    </i>
+    <i>
+      <x v="15"/>
+    </i>
+    <i>
+      <x v="16"/>
+    </i>
+    <i>
+      <x v="17"/>
+    </i>
+    <i>
+      <x v="18"/>
+    </i>
+    <i>
+      <x v="19"/>
+    </i>
+    <i>
+      <x v="21"/>
+    </i>
+    <i>
+      <x v="22"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="17"/>
+  </colFields>
+  <colItems count="12">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of place_type_1" fld="19" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="2">
+    <format dxfId="104">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="17" count="0" selected="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="103">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="17" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight15" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable11.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{676D4B45-E5CD-5641-8482-88793E8E33FA}" name="PivotTable6" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="B4:C16" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="28">
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" dataField="1" showAll="0">
       <items count="12">
         <item x="8"/>
         <item x="5"/>
@@ -28319,82 +28524,15 @@
       <x/>
     </i>
   </rowItems>
-  <colFields count="1">
-    <field x="11"/>
-  </colFields>
-  <colItems count="11">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
+  <colItems count="1">
+    <i/>
   </colItems>
   <dataFields count="1">
-    <dataField name="Count of period" fld="11" subtotal="count" baseField="0" baseItem="0"/>
+    <dataField name="Count of historical_theme" fld="17" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
-  <formats count="5">
-    <format dxfId="101">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
-        <references count="1">
-          <reference field="11" count="0" selected="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="100">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="11" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="99">
-      <pivotArea dataOnly="0" grandCol="1" outline="0" axis="axisCol" fieldPosition="0"/>
-    </format>
-    <format dxfId="98">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="11" count="1">
-            <x v="9"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="97">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="11" count="1">
-            <x v="9"/>
-          </reference>
-        </references>
-      </pivotArea>
+  <formats count="1">
+    <format dxfId="105">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
   <pivotTableStyleInfo name="PivotStyleLight15" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
@@ -28409,390 +28547,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable11.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B437B2B5-1664-2548-85F6-6CECF3005C22}" name="PivotTable7" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
-  <location ref="E4:K17" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="28">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="12">
-        <item x="8"/>
-        <item x="5"/>
-        <item x="0"/>
-        <item x="6"/>
-        <item x="1"/>
-        <item x="10"/>
-        <item x="9"/>
-        <item x="2"/>
-        <item x="7"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisCol" dataField="1" showAll="0">
-      <items count="8">
-        <item m="1" x="5"/>
-        <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="4"/>
-        <item x="3"/>
-        <item m="1" x="6"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="17"/>
-  </rowFields>
-  <rowItems count="12">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i>
-      <x v="10"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="18"/>
-  </colFields>
-  <colItems count="6">
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Count of place_category" fld="18" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <formats count="4">
-    <format dxfId="105">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
-        <references count="1">
-          <reference field="18" count="0" selected="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="104">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="18" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="103">
-      <pivotArea grandCol="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="102">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="5">
-    <chartFormat chart="0" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="18" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="1" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="18" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="18" count="1" selected="0">
-            <x v="3"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="3" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="18" count="1" selected="0">
-            <x v="4"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="4" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="18" count="1" selected="0">
-            <x v="5"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight15" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
 <file path=xl/pivotTables/pivotTable12.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3D62713B-9F8A-E840-BABA-5B517B1740F0}" name="PivotTable2" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="18">
-  <location ref="A4:C10" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="28">
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField axis="axisRow" dataField="1" compact="0" outline="0" showAll="0" sortType="ascending">
-      <items count="8">
-        <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="4"/>
-        <item x="3"/>
-        <item h="1" m="1" x="6"/>
-        <item h="1" m="1" x="5"/>
-        <item t="default"/>
-      </items>
-      <autoSortScope>
-        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
-          <references count="1">
-            <reference field="4294967294" count="1" selected="0">
-              <x v="0"/>
-            </reference>
-          </references>
-        </pivotArea>
-      </autoSortScope>
-    </pivotField>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField compact="0" outline="0" dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField compact="0" outline="0" dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField compact="0" outline="0" dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField compact="0" outline="0" dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField compact="0" outline="0" dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="18"/>
-  </rowFields>
-  <rowItems count="6">
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="-2"/>
-  </colFields>
-  <colItems count="2">
-    <i>
-      <x/>
-    </i>
-    <i i="1">
-      <x v="1"/>
-    </i>
-  </colItems>
-  <dataFields count="2">
-    <dataField name="Count " fld="18" subtotal="count" baseField="0" baseItem="0"/>
-    <dataField name="Count of place_category" fld="18" subtotal="count" showDataAs="percentOfTotal" baseField="18" baseItem="0" numFmtId="10"/>
-  </dataFields>
-  <formats count="5">
-    <format dxfId="77">
-      <pivotArea dataOnly="0" outline="0" axis="axisValues" fieldPosition="0"/>
-    </format>
-    <format dxfId="76">
-      <pivotArea outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="18" count="0" selected="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="75">
-      <pivotArea outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="74">
-      <pivotArea outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="73">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="18" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-  </formats>
-  <chartFormats count="2">
-    <chartFormat chart="1" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="1" format="1" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight15" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable13.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{EB548357-F74C-8444-A768-CDAE66F1A87F}" name="PivotTable1" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="5">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{EB548357-F74C-8444-A768-CDAE66F1A87F}" name="PivotTable1" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="5">
   <location ref="A15:C21" firstHeaderRow="1" firstDataRow="1" firstDataCol="2"/>
   <pivotFields count="28">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -28974,14 +28730,14 @@
     <dataField name="Count of place_category" fld="18" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="14">
-    <format dxfId="91">
+    <format dxfId="86">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="18" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="90">
+    <format dxfId="85">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="18" count="4" defaultSubtotal="1">
@@ -28993,7 +28749,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="89">
+    <format dxfId="84">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="12" count="38">
@@ -29042,7 +28798,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="88">
+    <format dxfId="83">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="12" count="36">
@@ -29089,7 +28845,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="87">
+    <format dxfId="82">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="12" count="21">
@@ -29121,7 +28877,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="86">
+    <format dxfId="81">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="12" count="15">
@@ -29147,27 +28903,27 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="85">
+    <format dxfId="80">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="84">
+    <format dxfId="79">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="83">
+    <format dxfId="78">
       <pivotArea outline="0" fieldPosition="0">
         <references count="1">
           <reference field="18" count="0" selected="0" defaultSubtotal="1"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="82">
+    <format dxfId="77">
       <pivotArea outline="0" fieldPosition="0">
         <references count="1">
           <reference field="18" count="0" selected="0" defaultSubtotal="1"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="81">
+    <format dxfId="76">
       <pivotArea outline="0" fieldPosition="0">
         <references count="2">
           <reference field="12" count="1" selected="0">
@@ -29179,7 +28935,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="80">
+    <format dxfId="75">
       <pivotArea outline="0" fieldPosition="0">
         <references count="2">
           <reference field="12" count="1" selected="0">
@@ -29191,7 +28947,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="79">
+    <format dxfId="74">
       <pivotArea outline="0" fieldPosition="0">
         <references count="2">
           <reference field="12" count="1" selected="0">
@@ -29203,7 +28959,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="78">
+    <format dxfId="73">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="12" count="1">
@@ -29509,8 +29265,168 @@
 </pivotTableDefinition>
 </file>
 
+<file path=xl/pivotTables/pivotTable13.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3D62713B-9F8A-E840-BABA-5B517B1740F0}" name="PivotTable2" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="18">
+  <location ref="A4:C10" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="28">
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField axis="axisRow" dataField="1" compact="0" outline="0" showAll="0" sortType="ascending">
+      <items count="8">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item h="1" m="1" x="6"/>
+        <item h="1" m="1" x="5"/>
+        <item t="default"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="1">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField compact="0" outline="0" dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField compact="0" outline="0" dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField compact="0" outline="0" dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField compact="0" outline="0" dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField compact="0" outline="0" dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="18"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
+  </colItems>
+  <dataFields count="2">
+    <dataField name="Count " fld="18" subtotal="count" baseField="0" baseItem="0"/>
+    <dataField name="Count of place_category" fld="18" subtotal="count" showDataAs="percentOfTotal" baseField="18" baseItem="0" numFmtId="10"/>
+  </dataFields>
+  <formats count="5">
+    <format dxfId="91">
+      <pivotArea dataOnly="0" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+    <format dxfId="90">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="18" count="0" selected="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="89">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="88">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="87">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="18" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+  </formats>
+  <chartFormats count="2">
+    <chartFormat chart="1" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="1" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight15" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
 <file path=xl/pivotTables/pivotTable14.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{431073AF-99BD-6544-A074-24A523B00CC8}" name="PivotTable4" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" grandTotalCaption="Total" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="place_type">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{431073AF-99BD-6544-A074-24A523B00CC8}" name="PivotTable4" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" grandTotalCaption="Total" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="place_type">
   <location ref="B41:C45" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
@@ -29586,7 +29502,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable15.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E5D8018C-5317-064F-9916-EA9F94B674AB}" name="PivotTable3" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" grandTotalCaption="Total" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="place_type">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E5D8018C-5317-064F-9916-EA9F94B674AB}" name="PivotTable3" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" grandTotalCaption="Total" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="place_type">
   <location ref="B30:C37" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
@@ -29675,7 +29591,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable16.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00DFF08D-0B6E-6448-93FD-25831A6C2E07}" name="PivotTable2" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" grandTotalCaption="Total" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="place_type">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00DFF08D-0B6E-6448-93FD-25831A6C2E07}" name="PivotTable2" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" grandTotalCaption="Total" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="place_type">
   <location ref="B4:C26" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
@@ -29830,7 +29746,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable17.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A028AB9E-24FA-BC4C-9317-2B89AD171D85}" name="PivotTable17" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A028AB9E-24FA-BC4C-9317-2B89AD171D85}" name="PivotTable17" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A43:E48" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
@@ -29955,7 +29871,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable18.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{57812AA5-A583-8741-B532-B773D261C6C4}" name="PivotTable16" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{57812AA5-A583-8741-B532-B773D261C6C4}" name="PivotTable16" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A31:E39" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
@@ -30093,7 +30009,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable19.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3A250399-2A38-E74C-867B-89C57BE24D3D}" name="PivotTable5" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="4">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3A250399-2A38-E74C-867B-89C57BE24D3D}" name="PivotTable5" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="4">
   <location ref="A4:G27" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -30303,7 +30219,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D34AB9AC-D393-AD42-B429-1C5FBD2BDAA6}" name="PivotTable11" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="25">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D34AB9AC-D393-AD42-B429-1C5FBD2BDAA6}" name="PivotTable11" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="25">
   <location ref="B20:H32" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
@@ -30635,7 +30551,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable20.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3FAC62E4-CE0E-B448-B0AD-E9DAFC687FCC}" name="PivotTable1" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3FAC62E4-CE0E-B448-B0AD-E9DAFC687FCC}" name="PivotTable1" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A4:B88" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -31204,7 +31120,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable21.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{DC2A81C9-2295-5D4A-9D9E-67042CBE96DD}" name="PivotTable5" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{DC2A81C9-2295-5D4A-9D9E-67042CBE96DD}" name="PivotTable5" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="G4:H93" firstHeaderRow="1" firstDataRow="1" firstDataCol="2"/>
   <pivotFields count="28">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -31865,7 +31781,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable22.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{398DAB95-6B62-7542-991E-CC0B1911D56D}" name="PivotTable23" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="8" rowHeaderCaption="Ranking of coordinates precision">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{398DAB95-6B62-7542-991E-CC0B1911D56D}" name="PivotTable23" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="8" rowHeaderCaption="Ranking of coordinates precision">
   <location ref="B4:C9" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
@@ -32079,7 +31995,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable23.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{AF72CEC9-EB7F-CB4B-8771-70A8FC1B66DB}" name="PivotTable21" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{AF72CEC9-EB7F-CB4B-8771-70A8FC1B66DB}" name="PivotTable21" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
   <location ref="J4:O10" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
@@ -32444,7 +32360,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable24.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E7EF111F-433C-0D40-9BBB-6138C0E23072}" name="PivotTable2" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" grandTotalCaption="Total" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1" rowHeaderCaption="(filter on place_name)" colHeaderCaption="">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E7EF111F-433C-0D40-9BBB-6138C0E23072}" name="PivotTable2" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" grandTotalCaption="Total" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1" rowHeaderCaption="(filter on place_name)" colHeaderCaption="">
   <location ref="A3:G88" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
@@ -32931,7 +32847,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable25.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{755CB6A8-F227-BD4A-8C6B-B14AD47B09EF}" name="PivotTable1" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{755CB6A8-F227-BD4A-8C6B-B14AD47B09EF}" name="PivotTable1" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A2:M87" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
@@ -33422,7 +33338,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5B06BAFF-02CC-6045-8A5D-C7221D3A1BEA}" name="PivotTable10" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5B06BAFF-02CC-6045-8A5D-C7221D3A1BEA}" name="PivotTable10" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="B80:N92" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
@@ -33587,7 +33503,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{866A254B-AD3F-2D41-9122-CB764CF3D95B}" name="PivotTable2" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="14">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{866A254B-AD3F-2D41-9122-CB764CF3D95B}" name="PivotTable2" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="14">
   <location ref="B4:C15" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
@@ -33719,8 +33635,8 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{40E5F6EB-967C-394A-BAD8-4CA202DEDFD9}" name="PivotTable14" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="B74:N97" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B437B2B5-1664-2548-85F6-6CECF3005C22}" name="PivotTable7" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
+  <location ref="E4:K17" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
@@ -33739,7 +33655,7 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField axis="axisCol" showAll="0">
+    <pivotField axis="axisRow" showAll="0">
       <items count="12">
         <item x="8"/>
         <item x="5"/>
@@ -33755,226 +33671,18 @@
         <item t="default"/>
       </items>
     </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" dataField="1" showAll="0">
-      <items count="25">
+    <pivotField axis="axisCol" dataField="1" showAll="0">
+      <items count="8">
+        <item m="1" x="5"/>
+        <item x="2"/>
         <item x="0"/>
         <item x="1"/>
         <item x="4"/>
-        <item x="6"/>
-        <item m="1" x="21"/>
-        <item x="18"/>
-        <item x="13"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="17"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item x="16"/>
-        <item x="9"/>
         <item x="3"/>
-        <item x="14"/>
-        <item x="5"/>
-        <item x="2"/>
-        <item x="10"/>
-        <item x="19"/>
-        <item m="1" x="22"/>
-        <item x="15"/>
-        <item x="20"/>
-        <item m="1" x="23"/>
+        <item m="1" x="6"/>
         <item t="default"/>
       </items>
     </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="19"/>
-  </rowFields>
-  <rowItems count="22">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i>
-      <x v="10"/>
-    </i>
-    <i>
-      <x v="11"/>
-    </i>
-    <i>
-      <x v="12"/>
-    </i>
-    <i>
-      <x v="13"/>
-    </i>
-    <i>
-      <x v="14"/>
-    </i>
-    <i>
-      <x v="15"/>
-    </i>
-    <i>
-      <x v="16"/>
-    </i>
-    <i>
-      <x v="17"/>
-    </i>
-    <i>
-      <x v="18"/>
-    </i>
-    <i>
-      <x v="19"/>
-    </i>
-    <i>
-      <x v="21"/>
-    </i>
-    <i>
-      <x v="22"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="17"/>
-  </colFields>
-  <colItems count="12">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i>
-      <x v="10"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Count of place_type_1" fld="19" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <formats count="2">
-    <format dxfId="93">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
-        <references count="1">
-          <reference field="17" count="0" selected="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="92">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="17" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-  </formats>
-  <pivotTableStyleInfo name="PivotStyleLight15" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{676D4B45-E5CD-5641-8482-88793E8E33FA}" name="PivotTable6" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="B4:C16" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="28">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" dataField="1" showAll="0">
-      <items count="12">
-        <item x="8"/>
-        <item x="5"/>
-        <item x="0"/>
-        <item x="6"/>
-        <item x="1"/>
-        <item x="10"/>
-        <item x="9"/>
-        <item x="2"/>
-        <item x="7"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
@@ -34026,17 +33734,116 @@
       <x/>
     </i>
   </rowItems>
-  <colItems count="1">
-    <i/>
+  <colFields count="1">
+    <field x="18"/>
+  </colFields>
+  <colItems count="6">
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
   </colItems>
   <dataFields count="1">
-    <dataField name="Count of historical_theme" fld="17" subtotal="count" baseField="0" baseItem="0"/>
+    <dataField name="Count of place_category" fld="18" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
-  <formats count="1">
+  <formats count="4">
+    <format dxfId="95">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="18" count="0" selected="0"/>
+        </references>
+      </pivotArea>
+    </format>
     <format dxfId="94">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="18" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="93">
+      <pivotArea grandCol="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="92">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
+  <chartFormats count="5">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="18" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="18" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="18" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="3" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="18" count="1" selected="0">
+            <x v="4"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="4" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="18" count="1" selected="0">
+            <x v="5"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight15" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
@@ -34049,8 +33856,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{7F76D8A8-3873-CE44-9B15-DC7D401C95D2}" name="PivotTable1" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="24">
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{7F76D8A8-3873-CE44-9B15-DC7D401C95D2}" name="PivotTable1" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="24">
   <location ref="O4:P16" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
@@ -34145,10 +33952,10 @@
     <dataField name="% of historical_theme" fld="17" subtotal="count" showDataAs="percentOfTotal" baseField="0" baseItem="0" numFmtId="10"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="96">
+    <format dxfId="97">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="95">
+    <format dxfId="96">
       <pivotArea outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -34454,8 +34261,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A35914F5-E8F2-9942-90D9-D73227088057}" name="PivotTable5" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A35914F5-E8F2-9942-90D9-D73227088057}" name="PivotTable5" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="B38:M45" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
@@ -34588,8 +34395,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable9.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{83629486-73F7-2B4A-B03B-54E32B8FB999}" name="PivotTable9" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{83629486-73F7-2B4A-B03B-54E32B8FB999}" name="PivotTable9" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="B48:M71" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="28">
     <pivotField showAll="0"/>
@@ -34775,6 +34582,199 @@
   <dataFields count="1">
     <dataField name="Count of place_type_1" fld="19" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight15" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable9.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5D78F90B-4103-B24B-BC63-5828426FA314}" name="PivotTable8" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" grandTotalCaption="Grand Total" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+  <location ref="B22:M35" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="28">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisCol" dataField="1" showAll="0">
+      <items count="11">
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="4"/>
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item n="Unknown _x000a_1840-1900_x000a_" x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="12">
+        <item x="8"/>
+        <item x="5"/>
+        <item x="0"/>
+        <item x="6"/>
+        <item x="1"/>
+        <item x="10"/>
+        <item x="9"/>
+        <item x="2"/>
+        <item x="7"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="17"/>
+  </rowFields>
+  <rowItems count="12">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="11"/>
+  </colFields>
+  <colItems count="11">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of period" fld="11" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="5">
+    <format dxfId="102">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="11" count="0" selected="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="101">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="11" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="100">
+      <pivotArea dataOnly="0" grandCol="1" outline="0" axis="axisCol" fieldPosition="0"/>
+    </format>
+    <format dxfId="99">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="11" count="1">
+            <x v="9"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="98">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="11" count="1">
+            <x v="9"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+  </formats>
   <pivotTableStyleInfo name="PivotStyleLight15" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
@@ -35207,11 +35207,11 @@
   <sheetData>
     <row r="1" spans="1:11" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="1:11" ht="19" x14ac:dyDescent="0.25">
-      <c r="A2" s="97" t="s">
+      <c r="A2" s="100" t="s">
         <v>216</v>
       </c>
-      <c r="B2" s="98"/>
-      <c r="C2" s="99"/>
+      <c r="B2" s="101"/>
+      <c r="C2" s="102"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="21" t="s">
@@ -35303,8 +35303,8 @@
       <c r="C10" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="J10" s="100"/>
-      <c r="K10" s="100"/>
+      <c r="J10" s="103"/>
+      <c r="K10" s="103"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" s="27" t="s">
@@ -39282,15 +39282,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="D1" s="113" t="s">
+      <c r="D1" s="99" t="s">
         <v>646</v>
       </c>
-      <c r="E1" s="113"/>
-      <c r="H1" s="113" t="s">
+      <c r="E1" s="99"/>
+      <c r="H1" s="99" t="s">
         <v>633</v>
       </c>
-      <c r="I1" s="113"/>
-      <c r="J1" s="113"/>
+      <c r="I1" s="99"/>
+      <c r="J1" s="99"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
@@ -41391,13 +41391,13 @@
       </c>
     </row>
     <row r="4" spans="2:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="101" t="s">
+      <c r="B4" s="113" t="s">
         <v>1138</v>
       </c>
-      <c r="C4" s="111" t="s">
+      <c r="C4" s="112" t="s">
         <v>1277</v>
       </c>
-      <c r="D4" s="103" t="s">
+      <c r="D4" s="111" t="s">
         <v>1185</v>
       </c>
       <c r="F4" s="31"/>
@@ -41416,9 +41416,9 @@
       </c>
     </row>
     <row r="5" spans="2:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="101"/>
-      <c r="C5" s="111"/>
-      <c r="D5" s="103"/>
+      <c r="B5" s="113"/>
+      <c r="C5" s="112"/>
+      <c r="D5" s="111"/>
       <c r="F5" s="31"/>
       <c r="G5" s="31"/>
       <c r="H5" s="31" t="s">
@@ -41435,9 +41435,9 @@
       </c>
     </row>
     <row r="6" spans="2:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="101"/>
-      <c r="C6" s="111"/>
-      <c r="D6" s="103"/>
+      <c r="B6" s="113"/>
+      <c r="C6" s="112"/>
+      <c r="D6" s="111"/>
       <c r="F6" s="31"/>
       <c r="G6" s="31"/>
       <c r="H6" s="31" t="s">
@@ -41465,10 +41465,10 @@
       <c r="I7" s="32" t="s">
         <v>606</v>
       </c>
-      <c r="K7" s="100" t="s">
+      <c r="K7" s="103" t="s">
         <v>965</v>
       </c>
-      <c r="L7" s="100"/>
+      <c r="L7" s="103"/>
     </row>
     <row r="8" spans="2:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="72" t="s">
@@ -41551,13 +41551,13 @@
       </c>
     </row>
     <row r="12" spans="2:12" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="101" t="s">
+      <c r="B12" s="113" t="s">
         <v>1151</v>
       </c>
-      <c r="C12" s="102" t="s">
+      <c r="C12" s="114" t="s">
         <v>1283</v>
       </c>
-      <c r="D12" s="103" t="s">
+      <c r="D12" s="111" t="s">
         <v>1244</v>
       </c>
       <c r="F12" s="34" t="s">
@@ -41574,9 +41574,9 @@
       </c>
     </row>
     <row r="13" spans="2:12" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="101"/>
-      <c r="C13" s="102"/>
-      <c r="D13" s="103"/>
+      <c r="B13" s="113"/>
+      <c r="C13" s="114"/>
+      <c r="D13" s="111"/>
       <c r="F13" s="50" t="s">
         <v>3</v>
       </c>
@@ -41591,13 +41591,13 @@
       </c>
     </row>
     <row r="14" spans="2:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="104" t="s">
+      <c r="B14" s="115" t="s">
         <v>1139</v>
       </c>
-      <c r="C14" s="102" t="s">
+      <c r="C14" s="114" t="s">
         <v>1284</v>
       </c>
-      <c r="D14" s="103" t="s">
+      <c r="D14" s="111" t="s">
         <v>1241</v>
       </c>
       <c r="F14" s="28" t="s">
@@ -41614,9 +41614,9 @@
       </c>
     </row>
     <row r="15" spans="2:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="104"/>
-      <c r="C15" s="102"/>
-      <c r="D15" s="103"/>
+      <c r="B15" s="115"/>
+      <c r="C15" s="114"/>
+      <c r="D15" s="111"/>
       <c r="F15" s="28"/>
       <c r="G15" s="28"/>
       <c r="H15" s="28" t="s">
@@ -41685,10 +41685,10 @@
       </c>
     </row>
     <row r="20" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="114" t="s">
+      <c r="B20" s="104" t="s">
         <v>1321</v>
       </c>
-      <c r="C20" s="114"/>
+      <c r="C20" s="104"/>
       <c r="F20" s="28"/>
       <c r="G20" s="28"/>
       <c r="H20" s="28" t="s">
@@ -41699,10 +41699,10 @@
       </c>
     </row>
     <row r="21" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B21" s="116" t="s">
+      <c r="B21" s="98" t="s">
         <v>261</v>
       </c>
-      <c r="C21" s="116" t="s">
+      <c r="C21" s="98" t="s">
         <v>1322</v>
       </c>
       <c r="F21" s="28"/>
@@ -41715,7 +41715,7 @@
       </c>
     </row>
     <row r="22" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="115" t="s">
+      <c r="B22" s="97" t="s">
         <v>262</v>
       </c>
       <c r="C22" s="25" t="s">
@@ -41731,7 +41731,7 @@
       </c>
     </row>
     <row r="23" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B23" s="115" t="s">
+      <c r="B23" s="97" t="s">
         <v>1256</v>
       </c>
       <c r="C23" s="25" t="s">
@@ -41747,7 +41747,7 @@
       </c>
     </row>
     <row r="24" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="115" t="s">
+      <c r="B24" s="97" t="s">
         <v>1194</v>
       </c>
       <c r="C24" s="25" t="s">
@@ -41763,7 +41763,7 @@
       </c>
     </row>
     <row r="25" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="115" t="s">
+      <c r="B25" s="97" t="s">
         <v>1189</v>
       </c>
       <c r="C25" s="25" t="s">
@@ -41779,7 +41779,7 @@
       </c>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B26" s="115" t="s">
+      <c r="B26" s="97" t="s">
         <v>1190</v>
       </c>
       <c r="C26" s="25" t="s">
@@ -41787,7 +41787,7 @@
       </c>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B27" s="115" t="s">
+      <c r="B27" s="97" t="s">
         <v>1192</v>
       </c>
       <c r="C27" s="25" t="s">
@@ -41795,7 +41795,7 @@
       </c>
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B28" s="115" t="s">
+      <c r="B28" s="97" t="s">
         <v>1193</v>
       </c>
       <c r="C28" s="25" t="s">
@@ -41803,7 +41803,7 @@
       </c>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B29" s="115" t="s">
+      <c r="B29" s="97" t="s">
         <v>1191</v>
       </c>
       <c r="C29" s="25" t="s">
@@ -41811,7 +41811,7 @@
       </c>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B30" s="115">
+      <c r="B30" s="97">
         <v>1900</v>
       </c>
       <c r="C30" s="25" t="s">
@@ -41819,7 +41819,7 @@
       </c>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B31" s="115" t="s">
+      <c r="B31" s="97" t="s">
         <v>1197</v>
       </c>
       <c r="C31" s="25" t="s">
@@ -59888,10 +59888,10 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:33" x14ac:dyDescent="0.2">
-      <c r="B2" s="112" t="s">
+      <c r="B2" s="116" t="s">
         <v>1251</v>
       </c>
-      <c r="C2" s="112"/>
+      <c r="C2" s="116"/>
     </row>
     <row r="4" spans="2:33" x14ac:dyDescent="0.2">
       <c r="B4" s="11" t="s">

</xml_diff>